<commit_message>
feat：Secondary confirmation for sensitive operations
</commit_message>
<xml_diff>
--- a/移动应用开发大作业评分表.xlsx
+++ b/移动应用开发大作业评分表.xlsx
@@ -589,14 +589,14 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+    </font>
+    <font>
       <b/>
       <sz val="20"/>
-      <color rgb="FF000000"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-    </font>
-    <font>
-      <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="宋体"/>
       <charset val="0"/>
@@ -2022,7 +2022,9 @@
       <c r="C22" s="14">
         <v>3</v>
       </c>
-      <c r="D22" s="15"/>
+      <c r="D22" s="15">
+        <v>3</v>
+      </c>
     </row>
     <row r="23" ht="50" customHeight="1" spans="1:4">
       <c r="A23" s="25" t="s">
@@ -2092,7 +2094,9 @@
       <c r="C28" s="32">
         <v>4</v>
       </c>
-      <c r="D28" s="32"/>
+      <c r="D28" s="32">
+        <v>4</v>
+      </c>
     </row>
     <row r="29" ht="30" customHeight="1" spans="1:4">
       <c r="A29" s="25"/>
@@ -2102,7 +2106,9 @@
       <c r="C29" s="32">
         <v>3</v>
       </c>
-      <c r="D29" s="32"/>
+      <c r="D29" s="32">
+        <v>3</v>
+      </c>
     </row>
     <row r="30" ht="30" customHeight="1" spans="1:4">
       <c r="A30" s="25"/>
@@ -2112,7 +2118,9 @@
       <c r="C30" s="32">
         <v>2</v>
       </c>
-      <c r="D30" s="32"/>
+      <c r="D30" s="32">
+        <v>2</v>
+      </c>
     </row>
     <row r="31" ht="30" customHeight="1" spans="1:4">
       <c r="A31" s="33" t="s">
@@ -2261,7 +2269,7 @@
       </c>
       <c r="D48" s="44">
         <f>SUM(D8:D47)</f>
-        <v>41</v>
+        <v>53</v>
       </c>
     </row>
   </sheetData>

</xml_diff>